<commit_message>
Decks à finitions, deck Années 90, nettoyage des mentions de plateau
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q4e3JGtiCx8jxBb2JR7Gh3
</commit_message>
<xml_diff>
--- a/Connoisseur_modele_themes.xlsx
+++ b/Connoisseur_modele_themes.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thèmes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cartes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode d'emploi" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +449,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Catégorie</t>
+          <t>Deck</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -475,7 +476,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Insolite</t>
+          <t>Mon deck</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -651,11 +652,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Savoirs</t>
-        </is>
-      </c>
+      <c r="A12" s="2" t="inlineStr"/>
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Votre thème ici</t>
@@ -749,10 +746,7 @@
       <c r="E21" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="A2:A2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Savoirs,Vie d’adulte,Loisirs,Insolite"</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>10</formula2>
@@ -768,7 +762,65 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Deck</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Finition</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Mon deck</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Irisé</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Une phrase qui donne envie de jouer ce deck.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Irisé,Métal,Or,Cuivre,Nacre,Néon,Rétro,Bleu,Rouge,Jaune,Vert,Violet,Craie"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -787,49 +839,70 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>• Une ligne par question, 10 lignes par thème (niveaux 1 à 10, du plus facile au plus pointu).</t>
+          <t>• Une carte = un thème de 10 questions. Un deck = un paquet de cartes (ex. « Années 90 »).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>• Catégorie : Savoirs, Vie d’adulte, Loisirs ou Insolite (liste déroulante).</t>
+          <t>• Feuille « Cartes » : Deck, Thème, Niveau, Question, Réponse.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>• Catégorie et Thème peuvent rester vides sous la première ligne d’un thème : la valeur du dessus est reprise.</t>
+          <t>• Feuille « Decks » : le nom de chaque deck, sa finition et une courte description.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>• Un niveau manquant sera simplement grisé dans le jeu.</t>
+          <t>• Finitions : Irisé, Métal, Or, Cuivre, Nacre, Néon, Rétro, Bleu, Rouge, Jaune, Vert, Violet, Craie, ou un code couleur comme #ff6600.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>• Vous pouvez mettre plusieurs thèmes dans la même feuille, ou répartir sur plusieurs feuilles avec les mêmes colonnes.</t>
+          <t>• Une ligne par question, 10 lignes par thème (niveaux 1 à 10, du plus facile au plus pointu).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>• Réimporter un thème du même nom et de la même catégorie le met à jour.</t>
+          <t>• Deck et Thème peuvent rester vides sous la première ligne d’un thème : la valeur du dessus est reprise.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>• Supprimez l’exemple « Pigeons » et la ligne « Votre thème ici » si vous ne les voulez pas.</t>
+          <t>• Un niveau manquant sera simplement grisé dans le jeu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>• Vous pouvez mettre plusieurs thèmes dans la même feuille, ou répartir sur plusieurs feuilles avec les mêmes colonnes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>• Réimporter un thème du même nom dans le même deck le met à jour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>• Remplacez « Mon deck » par le nom de votre deck, et supprimez l’exemple « Pigeons » si vous n’en voulez pas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2 : 6 nouvelles finitions retenues dans le labo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q4e3JGtiCx8jxBb2JR7Gh3
</commit_message>
<xml_diff>
--- a/Connoisseur_modele_themes.xlsx
+++ b/Connoisseur_modele_themes.xlsx
@@ -807,7 +807,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Irisé,Métal,Or,Cuivre,Nacre,Néon,Rétro,Bleu,Rouge,Jaune,Vert,Violet,Craie"</formula1>
+      <formula1>"Irisé,Métal,Or,Cuivre,Nacre,Néon,Chrome bleu,Papier millimétré,Confettis,Synthwave,Années 70,Vaporwave,Rétro,Bleu,Rouge,Jaune,Vert,Violet,Craie"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -860,7 +860,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>• Finitions : Irisé, Métal, Or, Cuivre, Nacre, Néon, Rétro, Bleu, Rouge, Jaune, Vert, Violet, Craie, ou un code couleur comme #ff6600.</t>
+          <t>• Finitions : Irisé, Métal, Or, Cuivre, Chrome bleu, Nacre, Néon, Papier millimétré, Confettis, Synthwave, Années 70, Vaporwave, Rétro, Bleu, Rouge, Jaune, Vert, Violet, Craie, ou un code couleur comme #ff6600.</t>
         </is>
       </c>
     </row>

</xml_diff>